<commit_message>
Before updating the overall stage 2 script.
</commit_message>
<xml_diff>
--- a/results/01_pollution_assessment/HZD_Focus/tables/stressor_cutoff_metrics.xlsx
+++ b/results/01_pollution_assessment/HZD_Focus/tables/stressor_cutoff_metrics.xlsx
@@ -491,24 +491,28 @@
         <v>57</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>0.09486046556535253</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
+        <v>0.006121295522739989</v>
+      </c>
+      <c r="F2" t="n">
+        <v>1.068980761481098</v>
+      </c>
       <c r="G2" t="n">
-        <v>0.001</v>
+        <v>0.366</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>113.2402726323594</v>
       </c>
       <c r="I2" t="n">
         <v>1193.756239308613</v>
       </c>
-      <c r="J2" t="inlineStr"/>
+      <c r="J2" t="n">
+        <v>0.8587878016819933</v>
+      </c>
       <c r="K2" t="n">
-        <v>1</v>
+        <v>16.05323832208607</v>
       </c>
     </row>
     <row r="3">
@@ -522,24 +526,28 @@
         <v>57</v>
       </c>
       <c r="D3" t="n">
-        <v>0</v>
+        <v>0.09486046556535253</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F3" t="inlineStr"/>
+        <v>0.006121295522739989</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1.068980761481098</v>
+      </c>
       <c r="G3" t="n">
-        <v>0.001</v>
+        <v>0.339</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
+        <v>113.2402726323594</v>
       </c>
       <c r="I3" t="n">
         <v>1193.756239308613</v>
       </c>
-      <c r="J3" t="inlineStr"/>
+      <c r="J3" t="n">
+        <v>0.8587878016819933</v>
+      </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>16.05323832208607</v>
       </c>
     </row>
     <row r="4">
@@ -553,24 +561,28 @@
         <v>57</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>0.09486046556535253</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
-      </c>
-      <c r="F4" t="inlineStr"/>
+        <v>0.006121295522739989</v>
+      </c>
+      <c r="F4" t="n">
+        <v>1.068980761481098</v>
+      </c>
       <c r="G4" t="n">
-        <v>0.001</v>
+        <v>0.363</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>113.2402726323594</v>
       </c>
       <c r="I4" t="n">
         <v>1193.756239308613</v>
       </c>
-      <c r="J4" t="inlineStr"/>
+      <c r="J4" t="n">
+        <v>0.8587878016819933</v>
+      </c>
       <c r="K4" t="n">
-        <v>1</v>
+        <v>16.05323832208607</v>
       </c>
     </row>
     <row r="5">
@@ -584,24 +596,28 @@
         <v>57</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>0.09486046556535253</v>
       </c>
       <c r="E5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F5" t="inlineStr"/>
+        <v>0.006121295522739989</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1.068980761481098</v>
+      </c>
       <c r="G5" t="n">
-        <v>0.001</v>
+        <v>0.374</v>
       </c>
       <c r="H5" t="n">
-        <v>0</v>
+        <v>113.2402726323594</v>
       </c>
       <c r="I5" t="n">
         <v>1193.756239308613</v>
       </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="n">
+        <v>0.8587878016819933</v>
+      </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>16.05323832208607</v>
       </c>
     </row>
     <row r="6">
@@ -615,24 +631,28 @@
         <v>57</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>0.09486046556535253</v>
       </c>
       <c r="E6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F6" t="inlineStr"/>
+        <v>0.006121295522739989</v>
+      </c>
+      <c r="F6" t="n">
+        <v>1.068980761481098</v>
+      </c>
       <c r="G6" t="n">
-        <v>0.001</v>
+        <v>0.352</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>113.2402726323594</v>
       </c>
       <c r="I6" t="n">
         <v>1193.756239308613</v>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="n">
+        <v>0.8587878016819933</v>
+      </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>16.05323832208607</v>
       </c>
     </row>
     <row r="7">
@@ -646,24 +666,28 @@
         <v>57</v>
       </c>
       <c r="D7" t="n">
-        <v>0</v>
+        <v>0.09486046556535253</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="inlineStr"/>
+        <v>0.006121295522739989</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1.068980761481098</v>
+      </c>
       <c r="G7" t="n">
-        <v>0.001</v>
+        <v>0.349</v>
       </c>
       <c r="H7" t="n">
-        <v>0</v>
+        <v>113.2402726323594</v>
       </c>
       <c r="I7" t="n">
         <v>1193.756239308613</v>
       </c>
-      <c r="J7" t="inlineStr"/>
+      <c r="J7" t="n">
+        <v>0.8587878016819933</v>
+      </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>16.05323832208607</v>
       </c>
     </row>
     <row r="8">
@@ -677,24 +701,28 @@
         <v>57</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>0.09486046556535253</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="inlineStr"/>
+        <v>0.006121295522739989</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.068980761481098</v>
+      </c>
       <c r="G8" t="n">
-        <v>0.001</v>
+        <v>0.355</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>113.2402726323594</v>
       </c>
       <c r="I8" t="n">
         <v>1193.756239308613</v>
       </c>
-      <c r="J8" t="inlineStr"/>
+      <c r="J8" t="n">
+        <v>0.8587878016819933</v>
+      </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>16.05323832208607</v>
       </c>
     </row>
     <row r="9">
@@ -708,24 +736,28 @@
         <v>57</v>
       </c>
       <c r="D9" t="n">
-        <v>0</v>
+        <v>0.09486046556535253</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="inlineStr"/>
+        <v>0.006121295522739989</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.068980761481098</v>
+      </c>
       <c r="G9" t="n">
-        <v>0.001</v>
+        <v>0.374</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>113.2402726323594</v>
       </c>
       <c r="I9" t="n">
         <v>1193.756239308613</v>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>0.8587878016819933</v>
+      </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>16.05323832208607</v>
       </c>
     </row>
     <row r="10">
@@ -739,24 +771,28 @@
         <v>57</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>0.09486046556535253</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="inlineStr"/>
+        <v>0.006121295522739989</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1.068980761481098</v>
+      </c>
       <c r="G10" t="n">
-        <v>0.001</v>
+        <v>0.366</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>113.2402726323594</v>
       </c>
       <c r="I10" t="n">
         <v>1193.756239308613</v>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>0.8587878016819933</v>
+      </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>16.05323832208607</v>
       </c>
     </row>
     <row r="11">
@@ -770,24 +806,28 @@
         <v>57</v>
       </c>
       <c r="D11" t="n">
-        <v>0</v>
+        <v>0.09486046556535253</v>
       </c>
       <c r="E11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" t="inlineStr"/>
+        <v>0.006121295522739989</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1.068980761481098</v>
+      </c>
       <c r="G11" t="n">
-        <v>0.001</v>
+        <v>0.377</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>113.2402726323594</v>
       </c>
       <c r="I11" t="n">
         <v>1193.756239308613</v>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>0.8587878016819933</v>
+      </c>
       <c r="K11" t="n">
-        <v>1</v>
+        <v>16.05323832208607</v>
       </c>
     </row>
     <row r="12">
@@ -801,28 +841,28 @@
         <v>58</v>
       </c>
       <c r="D12" t="n">
-        <v>0.02269091255701996</v>
+        <v>0.09273371658976785</v>
       </c>
       <c r="E12" t="n">
-        <v>0.005238964566966819</v>
+        <v>0.005496573954168471</v>
       </c>
       <c r="F12" t="n">
-        <v>1.300193684392866</v>
+        <v>1.063007267181234</v>
       </c>
       <c r="G12" t="n">
-        <v>0.23</v>
+        <v>0.355</v>
       </c>
       <c r="H12" t="n">
-        <v>27.71632719738638</v>
+        <v>113.2716908045437</v>
       </c>
       <c r="I12" t="n">
         <v>1221.472566506</v>
       </c>
       <c r="J12" t="n">
-        <v>0.4862513543401121</v>
+        <v>0.8415333190615926</v>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>16.43949747034235</v>
       </c>
     </row>
     <row r="13">
@@ -836,28 +876,28 @@
         <v>62</v>
       </c>
       <c r="D13" t="n">
-        <v>0.02453033892644999</v>
+        <v>0.09461197743272624</v>
       </c>
       <c r="E13" t="n">
-        <v>0.008272511241890879</v>
+        <v>0.01377376113207684</v>
       </c>
       <c r="F13" t="n">
-        <v>1.50883250840133</v>
+        <v>1.170386752236716</v>
       </c>
       <c r="G13" t="n">
-        <v>0.126</v>
+        <v>0.213</v>
       </c>
       <c r="H13" t="n">
-        <v>32.45789024453138</v>
+        <v>125.1880452421424</v>
       </c>
       <c r="I13" t="n">
         <v>1323.17333004859</v>
       </c>
       <c r="J13" t="n">
-        <v>0.5320965613857604</v>
+        <v>0.7706659272543467</v>
       </c>
       <c r="K13" t="n">
-        <v>1</v>
+        <v>17.04541693731259</v>
       </c>
     </row>
     <row r="14">
@@ -871,28 +911,28 @@
         <v>67</v>
       </c>
       <c r="D14" t="n">
-        <v>0.01620875000947223</v>
+        <v>0.09124306910617572</v>
       </c>
       <c r="E14" t="n">
-        <v>0.001073500009617923</v>
+        <v>0.01675479608209174</v>
       </c>
       <c r="F14" t="n">
-        <v>1.070927140921246</v>
+        <v>1.224931998043162</v>
       </c>
       <c r="G14" t="n">
-        <v>0.351</v>
+        <v>0.163</v>
       </c>
       <c r="H14" t="n">
-        <v>23.367298642189</v>
+        <v>131.540312706897</v>
       </c>
       <c r="I14" t="n">
         <v>1441.647173812502</v>
       </c>
       <c r="J14" t="n">
-        <v>0.354049979427106</v>
+        <v>0.7924681245655415</v>
       </c>
       <c r="K14" t="n">
-        <v>1</v>
+        <v>16.13716869647616</v>
       </c>
     </row>
     <row r="15">
@@ -906,28 +946,28 @@
         <v>72</v>
       </c>
       <c r="D15" t="n">
-        <v>0.01460547295425601</v>
+        <v>0.08607162238681054</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0005284082821739311</v>
+        <v>0.01683462408278114</v>
       </c>
       <c r="F15" t="n">
-        <v>1.037536822802406</v>
+        <v>1.243144915220874</v>
       </c>
       <c r="G15" t="n">
-        <v>0.349</v>
+        <v>0.16</v>
       </c>
       <c r="H15" t="n">
-        <v>22.56871389911598</v>
+        <v>132.9998574208872</v>
       </c>
       <c r="I15" t="n">
         <v>1545.223079718175</v>
       </c>
       <c r="J15" t="n">
-        <v>0.3178692098467041</v>
+        <v>0.7639330538564986</v>
       </c>
       <c r="K15" t="n">
-        <v>1</v>
+        <v>17.19867257881291</v>
       </c>
     </row>
     <row r="16">
@@ -941,28 +981,28 @@
         <v>76</v>
       </c>
       <c r="D16" t="n">
-        <v>0.01247551195550653</v>
+        <v>0.08367076427450235</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.0008694135586082563</v>
+        <v>0.01821867600839544</v>
       </c>
       <c r="F16" t="n">
-        <v>0.9348506248544681</v>
+        <v>1.278351332876105</v>
       </c>
       <c r="G16" t="n">
-        <v>0.468</v>
+        <v>0.135</v>
       </c>
       <c r="H16" t="n">
-        <v>20.33865913189402</v>
+        <v>136.4073201928221</v>
       </c>
       <c r="I16" t="n">
         <v>1630.286532883871</v>
       </c>
       <c r="J16" t="n">
-        <v>0.271182121758587</v>
+        <v>0.8156189763234923</v>
       </c>
       <c r="K16" t="n">
-        <v>1</v>
+        <v>17.57972441155299</v>
       </c>
     </row>
     <row r="17">
@@ -976,28 +1016,28 @@
         <v>81</v>
       </c>
       <c r="D17" t="n">
-        <v>0.01650073871402433</v>
+        <v>0.09339040005370247</v>
       </c>
       <c r="E17" t="n">
-        <v>0.004051380976227148</v>
+        <v>0.03294976005728267</v>
       </c>
       <c r="F17" t="n">
-        <v>1.325428914611946</v>
+        <v>1.545159019812404</v>
       </c>
       <c r="G17" t="n">
-        <v>0.205</v>
+        <v>0.019</v>
       </c>
       <c r="H17" t="n">
-        <v>28.33363958879021</v>
+        <v>160.3619075505736</v>
       </c>
       <c r="I17" t="n">
         <v>1717.113402002351</v>
       </c>
       <c r="J17" t="n">
-        <v>0.3541704948598777</v>
+        <v>0.9613373341215894</v>
       </c>
       <c r="K17" t="n">
-        <v>1</v>
+        <v>20.63707056100617</v>
       </c>
     </row>
     <row r="18">
@@ -1011,28 +1051,28 @@
         <v>86</v>
       </c>
       <c r="D18" t="n">
-        <v>0.01372764539297056</v>
+        <v>0.09373505684960622</v>
       </c>
       <c r="E18" t="n">
-        <v>0.001986307838125034</v>
+        <v>0.03709349790270666</v>
       </c>
       <c r="F18" t="n">
-        <v>1.169172194296146</v>
+        <v>1.654881302569392</v>
       </c>
       <c r="G18" t="n">
-        <v>0.267</v>
+        <v>0.014</v>
       </c>
       <c r="H18" t="n">
-        <v>24.89531983682641</v>
+        <v>169.9901296539163</v>
       </c>
       <c r="I18" t="n">
         <v>1813.517112670642</v>
       </c>
       <c r="J18" t="n">
-        <v>0.2928861157273693</v>
+        <v>0.8604724793907259</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>23.33475827825195</v>
       </c>
     </row>
     <row r="19">
@@ -1046,28 +1086,28 @@
         <v>90</v>
       </c>
       <c r="D19" t="n">
-        <v>0.01250334781456195</v>
+        <v>0.1045073451699739</v>
       </c>
       <c r="E19" t="n">
-        <v>0.001281794948818304</v>
+        <v>0.05120421095390093</v>
       </c>
       <c r="F19" t="n">
-        <v>1.114226164966108</v>
+        <v>1.960622892198727</v>
       </c>
       <c r="G19" t="n">
-        <v>0.326</v>
+        <v>0.003</v>
       </c>
       <c r="H19" t="n">
-        <v>24.23803397751677</v>
+        <v>202.5899479641603</v>
       </c>
       <c r="I19" t="n">
         <v>1938.523532816395</v>
       </c>
       <c r="J19" t="n">
-        <v>0.2723374604215367</v>
+        <v>0.980813329071342</v>
       </c>
       <c r="K19" t="n">
-        <v>1</v>
+        <v>23.04062819040346</v>
       </c>
     </row>
     <row r="20">
@@ -1081,28 +1121,28 @@
         <v>95</v>
       </c>
       <c r="D20" t="n">
-        <v>0.006237432351329804</v>
+        <v>0.09692062113028689</v>
       </c>
       <c r="E20" t="n">
-        <v>-0.00444818665564517</v>
+        <v>0.04618582456457276</v>
       </c>
       <c r="F20" t="n">
-        <v>0.5837221360090018</v>
+        <v>1.910338223289228</v>
       </c>
       <c r="G20" t="n">
-        <v>0.82</v>
+        <v>0.003</v>
       </c>
       <c r="H20" t="n">
-        <v>12.82406472187948</v>
+        <v>199.2673023531185</v>
       </c>
       <c r="I20" t="n">
         <v>2055.984578196735</v>
       </c>
       <c r="J20" t="n">
-        <v>0.1364262204455263</v>
+        <v>0.9536072016569527</v>
       </c>
       <c r="K20" t="n">
-        <v>1</v>
+        <v>25.68298951084523</v>
       </c>
     </row>
     <row r="21">
@@ -1116,28 +1156,28 @@
         <v>100</v>
       </c>
       <c r="D21" t="n">
-        <v>0.0102538231992958</v>
+        <v>0.09498735177881684</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0001543724156152226</v>
+        <v>0.046848381128754</v>
       </c>
       <c r="F21" t="n">
-        <v>1.015285228763587</v>
+        <v>1.973190338225329</v>
       </c>
       <c r="G21" t="n">
-        <v>0.401</v>
+        <v>0.002</v>
       </c>
       <c r="H21" t="n">
-        <v>21.87719381121574</v>
+        <v>202.6616476693315</v>
       </c>
       <c r="I21" t="n">
         <v>2133.564562798214</v>
       </c>
       <c r="J21" t="n">
-        <v>0.220981755668846</v>
+        <v>0.8767115730616204</v>
       </c>
       <c r="K21" t="n">
-        <v>1</v>
+        <v>26.17257829096286</v>
       </c>
     </row>
     <row r="22">
@@ -1151,25 +1191,25 @@
         <v>233</v>
       </c>
       <c r="D22" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E22" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F22" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G22" t="n">
         <v>0.001</v>
       </c>
       <c r="H22" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I22" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J22" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K22" t="n">
         <v>1</v>
@@ -1186,25 +1226,25 @@
         <v>233</v>
       </c>
       <c r="D23" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E23" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F23" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G23" t="n">
         <v>0.001</v>
       </c>
       <c r="H23" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I23" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J23" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K23" t="n">
         <v>1</v>
@@ -1221,25 +1261,25 @@
         <v>233</v>
       </c>
       <c r="D24" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E24" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F24" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G24" t="n">
         <v>0.001</v>
       </c>
       <c r="H24" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I24" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J24" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K24" t="n">
         <v>1</v>
@@ -1256,25 +1296,25 @@
         <v>233</v>
       </c>
       <c r="D25" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E25" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F25" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G25" t="n">
         <v>0.001</v>
       </c>
       <c r="H25" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I25" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J25" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K25" t="n">
         <v>1</v>
@@ -1291,25 +1331,25 @@
         <v>233</v>
       </c>
       <c r="D26" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E26" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F26" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G26" t="n">
         <v>0.001</v>
       </c>
       <c r="H26" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I26" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J26" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K26" t="n">
         <v>1</v>
@@ -1326,25 +1366,25 @@
         <v>233</v>
       </c>
       <c r="D27" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E27" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F27" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G27" t="n">
         <v>0.001</v>
       </c>
       <c r="H27" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I27" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J27" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K27" t="n">
         <v>1</v>
@@ -1361,25 +1401,25 @@
         <v>233</v>
       </c>
       <c r="D28" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E28" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F28" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G28" t="n">
         <v>0.001</v>
       </c>
       <c r="H28" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I28" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J28" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K28" t="n">
         <v>1</v>
@@ -1396,25 +1436,25 @@
         <v>233</v>
       </c>
       <c r="D29" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E29" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F29" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G29" t="n">
         <v>0.001</v>
       </c>
       <c r="H29" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I29" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J29" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K29" t="n">
         <v>1</v>
@@ -1431,25 +1471,25 @@
         <v>233</v>
       </c>
       <c r="D30" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E30" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F30" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G30" t="n">
         <v>0.001</v>
       </c>
       <c r="H30" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I30" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J30" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K30" t="n">
         <v>1</v>
@@ -1466,25 +1506,25 @@
         <v>233</v>
       </c>
       <c r="D31" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E31" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F31" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G31" t="n">
         <v>0.001</v>
       </c>
       <c r="H31" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I31" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J31" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K31" t="n">
         <v>1</v>
@@ -1501,25 +1541,25 @@
         <v>233</v>
       </c>
       <c r="D32" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E32" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F32" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G32" t="n">
         <v>0.001</v>
       </c>
       <c r="H32" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I32" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J32" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K32" t="n">
         <v>1</v>
@@ -1536,25 +1576,25 @@
         <v>233</v>
       </c>
       <c r="D33" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E33" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F33" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G33" t="n">
         <v>0.001</v>
       </c>
       <c r="H33" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I33" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J33" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K33" t="n">
         <v>1</v>
@@ -1571,25 +1611,25 @@
         <v>233</v>
       </c>
       <c r="D34" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E34" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F34" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G34" t="n">
         <v>0.001</v>
       </c>
       <c r="H34" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I34" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J34" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K34" t="n">
         <v>1</v>
@@ -1606,25 +1646,25 @@
         <v>233</v>
       </c>
       <c r="D35" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E35" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F35" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G35" t="n">
         <v>0.001</v>
       </c>
       <c r="H35" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I35" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J35" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K35" t="n">
         <v>1</v>
@@ -1641,25 +1681,25 @@
         <v>233</v>
       </c>
       <c r="D36" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E36" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F36" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G36" t="n">
         <v>0.001</v>
       </c>
       <c r="H36" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I36" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J36" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K36" t="n">
         <v>1</v>
@@ -1676,25 +1716,25 @@
         <v>233</v>
       </c>
       <c r="D37" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E37" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F37" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G37" t="n">
         <v>0.001</v>
       </c>
       <c r="H37" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I37" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J37" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K37" t="n">
         <v>1</v>
@@ -1711,25 +1751,25 @@
         <v>233</v>
       </c>
       <c r="D38" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E38" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F38" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G38" t="n">
         <v>0.001</v>
       </c>
       <c r="H38" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I38" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J38" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K38" t="n">
         <v>1</v>
@@ -1746,25 +1786,25 @@
         <v>233</v>
       </c>
       <c r="D39" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E39" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F39" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G39" t="n">
         <v>0.001</v>
       </c>
       <c r="H39" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I39" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J39" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K39" t="n">
         <v>1</v>
@@ -1781,25 +1821,25 @@
         <v>233</v>
       </c>
       <c r="D40" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E40" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F40" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G40" t="n">
         <v>0.001</v>
       </c>
       <c r="H40" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I40" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J40" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K40" t="n">
         <v>1</v>
@@ -1816,25 +1856,25 @@
         <v>233</v>
       </c>
       <c r="D41" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E41" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F41" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G41" t="n">
         <v>0.001</v>
       </c>
       <c r="H41" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I41" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J41" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K41" t="n">
         <v>1</v>
@@ -1851,25 +1891,25 @@
         <v>233</v>
       </c>
       <c r="D42" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E42" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F42" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G42" t="n">
         <v>0.001</v>
       </c>
       <c r="H42" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I42" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J42" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K42" t="n">
         <v>1</v>
@@ -1886,25 +1926,25 @@
         <v>233</v>
       </c>
       <c r="D43" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E43" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F43" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G43" t="n">
         <v>0.001</v>
       </c>
       <c r="H43" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I43" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J43" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K43" t="n">
         <v>1</v>
@@ -1921,25 +1961,25 @@
         <v>233</v>
       </c>
       <c r="D44" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E44" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F44" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G44" t="n">
         <v>0.001</v>
       </c>
       <c r="H44" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I44" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J44" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K44" t="n">
         <v>1</v>
@@ -1956,25 +1996,25 @@
         <v>233</v>
       </c>
       <c r="D45" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E45" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F45" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G45" t="n">
         <v>0.001</v>
       </c>
       <c r="H45" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I45" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J45" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K45" t="n">
         <v>1</v>
@@ -1991,25 +2031,25 @@
         <v>233</v>
       </c>
       <c r="D46" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E46" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F46" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G46" t="n">
         <v>0.001</v>
       </c>
       <c r="H46" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I46" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J46" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K46" t="n">
         <v>1</v>
@@ -2026,25 +2066,25 @@
         <v>233</v>
       </c>
       <c r="D47" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E47" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F47" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G47" t="n">
         <v>0.001</v>
       </c>
       <c r="H47" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I47" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J47" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K47" t="n">
         <v>1</v>
@@ -2061,25 +2101,25 @@
         <v>233</v>
       </c>
       <c r="D48" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E48" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F48" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G48" t="n">
         <v>0.001</v>
       </c>
       <c r="H48" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I48" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J48" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K48" t="n">
         <v>1</v>
@@ -2096,25 +2136,25 @@
         <v>233</v>
       </c>
       <c r="D49" t="n">
-        <v>0.03494176044427086</v>
+        <v>0.1014110673239307</v>
       </c>
       <c r="E49" t="n">
-        <v>0.03076401914749283</v>
+        <v>0.08161835955573538</v>
       </c>
       <c r="F49" t="n">
-        <v>8.363792289201486</v>
+        <v>5.123658092243791</v>
       </c>
       <c r="G49" t="n">
         <v>0.001</v>
       </c>
       <c r="H49" t="n">
-        <v>213.860861192194</v>
+        <v>620.685904675744</v>
       </c>
       <c r="I49" t="n">
         <v>6120.49474534301</v>
       </c>
       <c r="J49" t="n">
-        <v>0.9218140568629059</v>
+        <v>1.574534992213807</v>
       </c>
       <c r="K49" t="n">
         <v>1</v>

</xml_diff>

<commit_message>
Added AU sweeping over sites and cluluster numbers.
</commit_message>
<xml_diff>
--- a/results/01_pollution_assessment/HZD_Focus/tables/stressor_cutoff_metrics.xlsx
+++ b/results/01_pollution_assessment/HZD_Focus/tables/stressor_cutoff_metrics.xlsx
@@ -491,28 +491,28 @@
         <v>73</v>
       </c>
       <c r="D2" t="n">
-        <v>0.2059772426470385</v>
+        <v>0.2059772426470382</v>
       </c>
       <c r="E2" t="n">
-        <v>0.1467218129938325</v>
+        <v>0.1467218129938321</v>
       </c>
       <c r="F2" t="n">
-        <v>3.476090610641514</v>
+        <v>3.476090610641509</v>
       </c>
       <c r="G2" t="n">
         <v>0.001</v>
       </c>
       <c r="H2" t="n">
-        <v>381.4027242004413</v>
+        <v>381.4027242004407</v>
       </c>
       <c r="I2" t="n">
         <v>1851.674094181419</v>
       </c>
       <c r="J2" t="n">
-        <v>4.098282586189645</v>
+        <v>4.098282586189635</v>
       </c>
       <c r="K2" t="n">
-        <v>3.257428671522138</v>
+        <v>7.618053298098457</v>
       </c>
     </row>
     <row r="3">
@@ -526,28 +526,28 @@
         <v>73</v>
       </c>
       <c r="D3" t="n">
-        <v>0.2059772426470385</v>
+        <v>0.2059772426470382</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1467218129938325</v>
+        <v>0.1467218129938321</v>
       </c>
       <c r="F3" t="n">
-        <v>3.476090610641514</v>
+        <v>3.476090610641509</v>
       </c>
       <c r="G3" t="n">
         <v>0.001</v>
       </c>
       <c r="H3" t="n">
-        <v>381.4027242004413</v>
+        <v>381.4027242004407</v>
       </c>
       <c r="I3" t="n">
         <v>1851.674094181419</v>
       </c>
       <c r="J3" t="n">
-        <v>4.098282586189645</v>
+        <v>4.098282586189635</v>
       </c>
       <c r="K3" t="n">
-        <v>3.257428671522138</v>
+        <v>7.618053298098457</v>
       </c>
     </row>
     <row r="4">
@@ -561,28 +561,28 @@
         <v>73</v>
       </c>
       <c r="D4" t="n">
-        <v>0.2059772426470385</v>
+        <v>0.2059772426470382</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1467218129938325</v>
+        <v>0.1467218129938321</v>
       </c>
       <c r="F4" t="n">
-        <v>3.476090610641514</v>
+        <v>3.476090610641509</v>
       </c>
       <c r="G4" t="n">
         <v>0.001</v>
       </c>
       <c r="H4" t="n">
-        <v>381.4027242004413</v>
+        <v>381.4027242004407</v>
       </c>
       <c r="I4" t="n">
         <v>1851.674094181419</v>
       </c>
       <c r="J4" t="n">
-        <v>4.098282586189645</v>
+        <v>4.098282586189635</v>
       </c>
       <c r="K4" t="n">
-        <v>3.257428671522138</v>
+        <v>7.618053298098457</v>
       </c>
     </row>
     <row r="5">
@@ -596,28 +596,28 @@
         <v>73</v>
       </c>
       <c r="D5" t="n">
-        <v>0.2059772426470385</v>
+        <v>0.2059772426470382</v>
       </c>
       <c r="E5" t="n">
-        <v>0.1467218129938325</v>
+        <v>0.1467218129938321</v>
       </c>
       <c r="F5" t="n">
-        <v>3.476090610641514</v>
+        <v>3.476090610641509</v>
       </c>
       <c r="G5" t="n">
         <v>0.001</v>
       </c>
       <c r="H5" t="n">
-        <v>381.4027242004413</v>
+        <v>381.4027242004407</v>
       </c>
       <c r="I5" t="n">
         <v>1851.674094181419</v>
       </c>
       <c r="J5" t="n">
-        <v>4.098282586189645</v>
+        <v>4.098282586189635</v>
       </c>
       <c r="K5" t="n">
-        <v>3.257428671522138</v>
+        <v>7.618053298098457</v>
       </c>
     </row>
     <row r="6">
@@ -631,28 +631,28 @@
         <v>73</v>
       </c>
       <c r="D6" t="n">
-        <v>0.2059772426470385</v>
+        <v>0.2059772426470382</v>
       </c>
       <c r="E6" t="n">
-        <v>0.1467218129938325</v>
+        <v>0.1467218129938321</v>
       </c>
       <c r="F6" t="n">
-        <v>3.476090610641514</v>
+        <v>3.476090610641509</v>
       </c>
       <c r="G6" t="n">
         <v>0.001</v>
       </c>
       <c r="H6" t="n">
-        <v>381.4027242004413</v>
+        <v>381.4027242004407</v>
       </c>
       <c r="I6" t="n">
         <v>1851.674094181419</v>
       </c>
       <c r="J6" t="n">
-        <v>4.098282586189645</v>
+        <v>4.098282586189635</v>
       </c>
       <c r="K6" t="n">
-        <v>3.257428671522138</v>
+        <v>7.618053298098457</v>
       </c>
     </row>
     <row r="7">
@@ -666,28 +666,28 @@
         <v>73</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2059772426470385</v>
+        <v>0.2059772426470382</v>
       </c>
       <c r="E7" t="n">
-        <v>0.1467218129938325</v>
+        <v>0.1467218129938321</v>
       </c>
       <c r="F7" t="n">
-        <v>3.476090610641514</v>
+        <v>3.476090610641509</v>
       </c>
       <c r="G7" t="n">
         <v>0.001</v>
       </c>
       <c r="H7" t="n">
-        <v>381.4027242004413</v>
+        <v>381.4027242004407</v>
       </c>
       <c r="I7" t="n">
         <v>1851.674094181419</v>
       </c>
       <c r="J7" t="n">
-        <v>4.098282586189645</v>
+        <v>4.098282586189635</v>
       </c>
       <c r="K7" t="n">
-        <v>3.257428671522138</v>
+        <v>7.618053298098457</v>
       </c>
     </row>
     <row r="8">
@@ -701,28 +701,28 @@
         <v>73</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2059772426470385</v>
+        <v>0.2059772426470382</v>
       </c>
       <c r="E8" t="n">
-        <v>0.1467218129938325</v>
+        <v>0.1467218129938321</v>
       </c>
       <c r="F8" t="n">
-        <v>3.476090610641514</v>
+        <v>3.476090610641509</v>
       </c>
       <c r="G8" t="n">
         <v>0.001</v>
       </c>
       <c r="H8" t="n">
-        <v>381.4027242004413</v>
+        <v>381.4027242004407</v>
       </c>
       <c r="I8" t="n">
         <v>1851.674094181419</v>
       </c>
       <c r="J8" t="n">
-        <v>4.098282586189645</v>
+        <v>4.098282586189635</v>
       </c>
       <c r="K8" t="n">
-        <v>3.257428671522138</v>
+        <v>7.618053298098457</v>
       </c>
     </row>
     <row r="9">
@@ -736,28 +736,28 @@
         <v>73</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2059772426470385</v>
+        <v>0.2059772426470382</v>
       </c>
       <c r="E9" t="n">
-        <v>0.1467218129938325</v>
+        <v>0.1467218129938321</v>
       </c>
       <c r="F9" t="n">
-        <v>3.476090610641514</v>
+        <v>3.476090610641509</v>
       </c>
       <c r="G9" t="n">
         <v>0.001</v>
       </c>
       <c r="H9" t="n">
-        <v>381.4027242004413</v>
+        <v>381.4027242004407</v>
       </c>
       <c r="I9" t="n">
         <v>1851.674094181419</v>
       </c>
       <c r="J9" t="n">
-        <v>4.098282586189645</v>
+        <v>4.098282586189635</v>
       </c>
       <c r="K9" t="n">
-        <v>3.257428671522138</v>
+        <v>7.618053298098457</v>
       </c>
     </row>
     <row r="10">
@@ -771,28 +771,28 @@
         <v>73</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2059772426470385</v>
+        <v>0.2059772426470382</v>
       </c>
       <c r="E10" t="n">
-        <v>0.1467218129938325</v>
+        <v>0.1467218129938321</v>
       </c>
       <c r="F10" t="n">
-        <v>3.476090610641514</v>
+        <v>3.476090610641509</v>
       </c>
       <c r="G10" t="n">
         <v>0.001</v>
       </c>
       <c r="H10" t="n">
-        <v>381.4027242004413</v>
+        <v>381.4027242004407</v>
       </c>
       <c r="I10" t="n">
         <v>1851.674094181419</v>
       </c>
       <c r="J10" t="n">
-        <v>4.098282586189645</v>
+        <v>4.098282586189635</v>
       </c>
       <c r="K10" t="n">
-        <v>3.257428671522138</v>
+        <v>7.618053298098457</v>
       </c>
     </row>
     <row r="11">
@@ -806,28 +806,28 @@
         <v>73</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2059772426470385</v>
+        <v>0.2059772426470382</v>
       </c>
       <c r="E11" t="n">
-        <v>0.1467218129938325</v>
+        <v>0.1467218129938321</v>
       </c>
       <c r="F11" t="n">
-        <v>3.476090610641514</v>
+        <v>3.476090610641509</v>
       </c>
       <c r="G11" t="n">
         <v>0.001</v>
       </c>
       <c r="H11" t="n">
-        <v>381.4027242004413</v>
+        <v>381.4027242004407</v>
       </c>
       <c r="I11" t="n">
         <v>1851.674094181419</v>
       </c>
       <c r="J11" t="n">
-        <v>4.098282586189645</v>
+        <v>4.098282586189635</v>
       </c>
       <c r="K11" t="n">
-        <v>3.257428671522138</v>
+        <v>7.618053298098457</v>
       </c>
     </row>
     <row r="12">
@@ -853,16 +853,16 @@
         <v>0.001</v>
       </c>
       <c r="H12" t="n">
-        <v>365.1706141008648</v>
+        <v>365.1706141008647</v>
       </c>
       <c r="I12" t="n">
         <v>1942.633980068581</v>
       </c>
       <c r="J12" t="n">
-        <v>3.668079660838305</v>
+        <v>3.668079660838304</v>
       </c>
       <c r="K12" t="n">
-        <v>3.427863304970906</v>
+        <v>8.34917488483414</v>
       </c>
     </row>
     <row r="13">
@@ -876,28 +876,28 @@
         <v>83</v>
       </c>
       <c r="D13" t="n">
-        <v>0.1895609603152558</v>
+        <v>0.1895609603152557</v>
       </c>
       <c r="E13" t="n">
         <v>0.1369350486474152</v>
       </c>
       <c r="F13" t="n">
-        <v>3.602046108231046</v>
+        <v>3.602046108231044</v>
       </c>
       <c r="G13" t="n">
         <v>0.001</v>
       </c>
       <c r="H13" t="n">
-        <v>398.1879144980711</v>
+        <v>398.1879144980709</v>
       </c>
       <c r="I13" t="n">
         <v>2100.579749310466</v>
       </c>
       <c r="J13" t="n">
-        <v>3.671719855765078</v>
+        <v>3.67171985576508</v>
       </c>
       <c r="K13" t="n">
-        <v>3.148523905387103</v>
+        <v>6.651354131394607</v>
       </c>
     </row>
     <row r="14">
@@ -911,7 +911,7 @@
         <v>89</v>
       </c>
       <c r="D14" t="n">
-        <v>0.1723141820514099</v>
+        <v>0.1723141820514098</v>
       </c>
       <c r="E14" t="n">
         <v>0.1224535906087236</v>
@@ -923,16 +923,16 @@
         <v>0.001</v>
       </c>
       <c r="H14" t="n">
-        <v>388.0327834197182</v>
+        <v>388.032783419718</v>
       </c>
       <c r="I14" t="n">
         <v>2251.89116067039</v>
       </c>
       <c r="J14" t="n">
-        <v>3.317540845574616</v>
+        <v>3.317540845574614</v>
       </c>
       <c r="K14" t="n">
-        <v>3.328515319583292</v>
+        <v>6.899563435338715</v>
       </c>
     </row>
     <row r="15">
@@ -946,28 +946,28 @@
         <v>96</v>
       </c>
       <c r="D15" t="n">
-        <v>0.1713530624226824</v>
+        <v>0.1713530624226826</v>
       </c>
       <c r="E15" t="n">
-        <v>0.1253171214461648</v>
+        <v>0.1253171214461649</v>
       </c>
       <c r="F15" t="n">
-        <v>3.722158356882235</v>
+        <v>3.722158356882237</v>
       </c>
       <c r="G15" t="n">
         <v>0.001</v>
       </c>
       <c r="H15" t="n">
-        <v>416.0643176057742</v>
+        <v>416.0643176057745</v>
       </c>
       <c r="I15" t="n">
         <v>2428.111360971502</v>
       </c>
       <c r="J15" t="n">
-        <v>3.344082886305435</v>
+        <v>3.344082886305437</v>
       </c>
       <c r="K15" t="n">
-        <v>3.440807935581242</v>
+        <v>7.062161287368077</v>
       </c>
     </row>
     <row r="16">
@@ -981,28 +981,28 @@
         <v>102</v>
       </c>
       <c r="D16" t="n">
-        <v>0.1778821052081558</v>
+        <v>0.1778821052081557</v>
       </c>
       <c r="E16" t="n">
-        <v>0.135063464854414</v>
+        <v>0.1350634648544139</v>
       </c>
       <c r="F16" t="n">
-        <v>4.154314656855068</v>
+        <v>4.154314656855065</v>
       </c>
       <c r="G16" t="n">
         <v>0.001</v>
       </c>
       <c r="H16" t="n">
-        <v>457.0325838396894</v>
+        <v>457.0325838396891</v>
       </c>
       <c r="I16" t="n">
         <v>2569.30051117213</v>
       </c>
       <c r="J16" t="n">
-        <v>3.53643361223686</v>
+        <v>3.536433612236856</v>
       </c>
       <c r="K16" t="n">
-        <v>3.590532157936295</v>
+        <v>7.088105405133867</v>
       </c>
     </row>
     <row r="17">
@@ -1016,28 +1016,28 @@
         <v>108</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1816345347101616</v>
+        <v>0.1816345347101615</v>
       </c>
       <c r="E17" t="n">
-        <v>0.1415185805292872</v>
+        <v>0.141518580529287</v>
       </c>
       <c r="F17" t="n">
-        <v>4.527738113649487</v>
+        <v>4.527738113649484</v>
       </c>
       <c r="G17" t="n">
         <v>0.001</v>
       </c>
       <c r="H17" t="n">
-        <v>497.1237539218122</v>
+        <v>497.1237539218117</v>
       </c>
       <c r="I17" t="n">
         <v>2736.945122881416</v>
       </c>
       <c r="J17" t="n">
-        <v>3.571490106711147</v>
+        <v>3.571490106711145</v>
       </c>
       <c r="K17" t="n">
-        <v>3.730483117207455</v>
+        <v>7.396026412518752</v>
       </c>
     </row>
     <row r="18">
@@ -1051,28 +1051,28 @@
         <v>114</v>
       </c>
       <c r="D18" t="n">
-        <v>0.1815120186352368</v>
+        <v>0.1815120186352366</v>
       </c>
       <c r="E18" t="n">
-        <v>0.1436190565350163</v>
+        <v>0.1436190565350161</v>
       </c>
       <c r="F18" t="n">
-        <v>4.790124829913482</v>
+        <v>4.790124829913474</v>
       </c>
       <c r="G18" t="n">
         <v>0.001</v>
       </c>
       <c r="H18" t="n">
-        <v>519.1722281443733</v>
+        <v>519.1722281443725</v>
       </c>
       <c r="I18" t="n">
         <v>2860.26364561397</v>
       </c>
       <c r="J18" t="n">
-        <v>3.403827239368157</v>
+        <v>3.403827239368145</v>
       </c>
       <c r="K18" t="n">
-        <v>3.855027137717347</v>
+        <v>7.302291552842163</v>
       </c>
     </row>
     <row r="19">
@@ -1086,28 +1086,28 @@
         <v>120</v>
       </c>
       <c r="D19" t="n">
-        <v>0.1745212416838252</v>
+        <v>0.1745212416838254</v>
       </c>
       <c r="E19" t="n">
-        <v>0.1383160329857474</v>
+        <v>0.1383160329857476</v>
       </c>
       <c r="F19" t="n">
-        <v>4.820335193733896</v>
+        <v>4.820335193733901</v>
       </c>
       <c r="G19" t="n">
         <v>0.001</v>
       </c>
       <c r="H19" t="n">
-        <v>519.9667364455968</v>
+        <v>519.9667364455973</v>
       </c>
       <c r="I19" t="n">
         <v>2979.38939368541</v>
       </c>
       <c r="J19" t="n">
-        <v>3.204997495329263</v>
+        <v>3.204997495329267</v>
       </c>
       <c r="K19" t="n">
-        <v>3.953936295852069</v>
+        <v>7.618825632005373</v>
       </c>
     </row>
     <row r="20">
@@ -1121,28 +1121,28 @@
         <v>127</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1770269462939102</v>
+        <v>0.1770269462939107</v>
       </c>
       <c r="E20" t="n">
-        <v>0.1430197953143197</v>
+        <v>0.1430197953143202</v>
       </c>
       <c r="F20" t="n">
-        <v>5.205580038155907</v>
+        <v>5.205580038155918</v>
       </c>
       <c r="G20" t="n">
         <v>0.001</v>
       </c>
       <c r="H20" t="n">
-        <v>555.5491095556861</v>
+        <v>555.5491095556873</v>
       </c>
       <c r="I20" t="n">
         <v>3138.217775238193</v>
       </c>
       <c r="J20" t="n">
-        <v>3.223479395458611</v>
+        <v>3.223479395458619</v>
       </c>
       <c r="K20" t="n">
-        <v>3.606020413782225</v>
+        <v>6.396613824988021</v>
       </c>
     </row>
     <row r="21">
@@ -1156,28 +1156,28 @@
         <v>133</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1671951700237239</v>
+        <v>0.1671951700237238</v>
       </c>
       <c r="E21" t="n">
-        <v>0.1344075782923746</v>
+        <v>0.1344075782923745</v>
       </c>
       <c r="F21" t="n">
-        <v>5.099342806073259</v>
+        <v>5.099342806073256</v>
       </c>
       <c r="G21" t="n">
         <v>0.001</v>
       </c>
       <c r="H21" t="n">
-        <v>557.963480535009</v>
+        <v>557.9634805350087</v>
       </c>
       <c r="I21" t="n">
         <v>3337.198559359325</v>
       </c>
       <c r="J21" t="n">
-        <v>3.13149463621279</v>
+        <v>3.131494636212788</v>
       </c>
       <c r="K21" t="n">
-        <v>3.830513814545031</v>
+        <v>6.318823769436523</v>
       </c>
     </row>
     <row r="22">
@@ -1194,25 +1194,25 @@
         <v>0.1653376034645286</v>
       </c>
       <c r="E22" t="n">
-        <v>0.1339593178804882</v>
+        <v>0.1339593178804883</v>
       </c>
       <c r="F22" t="n">
-        <v>5.269172626455509</v>
+        <v>5.26917262645551</v>
       </c>
       <c r="G22" t="n">
         <v>0.001</v>
       </c>
       <c r="H22" t="n">
-        <v>565.0338114029144</v>
+        <v>565.0338114029145</v>
       </c>
       <c r="I22" t="n">
         <v>3417.454950132602</v>
       </c>
       <c r="J22" t="n">
-        <v>3.004821897171264</v>
+        <v>3.004821897171262</v>
       </c>
       <c r="K22" t="n">
-        <v>3.808328218021247</v>
+        <v>6.983521941156175</v>
       </c>
     </row>
     <row r="23">
@@ -1226,28 +1226,28 @@
         <v>145</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1595885382031379</v>
+        <v>0.1595885382031378</v>
       </c>
       <c r="E23" t="n">
-        <v>0.1293579100809487</v>
+        <v>0.1293579100809485</v>
       </c>
       <c r="F23" t="n">
-        <v>5.279034810593296</v>
+        <v>5.279034810593294</v>
       </c>
       <c r="G23" t="n">
         <v>0.001</v>
       </c>
       <c r="H23" t="n">
-        <v>560.292697363376</v>
+        <v>560.2926973633757</v>
       </c>
       <c r="I23" t="n">
         <v>3510.85800817467</v>
       </c>
       <c r="J23" t="n">
-        <v>2.74478706296467</v>
+        <v>2.744787062964669</v>
       </c>
       <c r="K23" t="n">
-        <v>4.08419358166231</v>
+        <v>7.1407644224968</v>
       </c>
     </row>
     <row r="24">
@@ -1261,28 +1261,28 @@
         <v>151</v>
       </c>
       <c r="D24" t="n">
-        <v>0.1609592739334942</v>
+        <v>0.160959273933494</v>
       </c>
       <c r="E24" t="n">
-        <v>0.1320268351036146</v>
+        <v>0.1320268351036143</v>
       </c>
       <c r="F24" t="n">
-        <v>5.56328054056978</v>
+        <v>5.563280540569773</v>
       </c>
       <c r="G24" t="n">
         <v>0.001</v>
       </c>
       <c r="H24" t="n">
-        <v>584.0607510682651</v>
+        <v>584.0607510682644</v>
       </c>
       <c r="I24" t="n">
         <v>3628.624414083713</v>
       </c>
       <c r="J24" t="n">
-        <v>2.646026079979103</v>
+        <v>2.646026079979099</v>
       </c>
       <c r="K24" t="n">
-        <v>4.16835008382468</v>
+        <v>7.171217634077469</v>
       </c>
     </row>
     <row r="25">
@@ -1296,28 +1296,28 @@
         <v>310</v>
       </c>
       <c r="D25" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E25" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F25" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G25" t="n">
         <v>0.001</v>
       </c>
       <c r="H25" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I25" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J25" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K25" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="26">
@@ -1331,28 +1331,28 @@
         <v>310</v>
       </c>
       <c r="D26" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E26" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F26" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G26" t="n">
         <v>0.001</v>
       </c>
       <c r="H26" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I26" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J26" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K26" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="27">
@@ -1366,28 +1366,28 @@
         <v>310</v>
       </c>
       <c r="D27" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E27" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F27" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G27" t="n">
         <v>0.001</v>
       </c>
       <c r="H27" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I27" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J27" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K27" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="28">
@@ -1401,28 +1401,28 @@
         <v>310</v>
       </c>
       <c r="D28" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E28" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F28" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G28" t="n">
         <v>0.001</v>
       </c>
       <c r="H28" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I28" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J28" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K28" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="29">
@@ -1436,28 +1436,28 @@
         <v>310</v>
       </c>
       <c r="D29" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E29" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F29" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G29" t="n">
         <v>0.001</v>
       </c>
       <c r="H29" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I29" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J29" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K29" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="30">
@@ -1471,28 +1471,28 @@
         <v>310</v>
       </c>
       <c r="D30" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E30" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F30" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G30" t="n">
         <v>0.001</v>
       </c>
       <c r="H30" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I30" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J30" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K30" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="31">
@@ -1506,28 +1506,28 @@
         <v>310</v>
       </c>
       <c r="D31" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E31" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F31" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G31" t="n">
         <v>0.001</v>
       </c>
       <c r="H31" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I31" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J31" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K31" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="32">
@@ -1541,28 +1541,28 @@
         <v>310</v>
       </c>
       <c r="D32" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E32" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F32" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G32" t="n">
         <v>0.001</v>
       </c>
       <c r="H32" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I32" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J32" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K32" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="33">
@@ -1576,28 +1576,28 @@
         <v>310</v>
       </c>
       <c r="D33" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E33" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F33" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G33" t="n">
         <v>0.001</v>
       </c>
       <c r="H33" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I33" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J33" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="34">
@@ -1611,28 +1611,28 @@
         <v>310</v>
       </c>
       <c r="D34" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E34" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F34" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G34" t="n">
         <v>0.001</v>
       </c>
       <c r="H34" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I34" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J34" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K34" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="35">
@@ -1646,28 +1646,28 @@
         <v>310</v>
       </c>
       <c r="D35" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E35" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F35" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G35" t="n">
         <v>0.001</v>
       </c>
       <c r="H35" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I35" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J35" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K35" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="36">
@@ -1681,28 +1681,28 @@
         <v>310</v>
       </c>
       <c r="D36" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E36" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F36" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G36" t="n">
         <v>0.001</v>
       </c>
       <c r="H36" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I36" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J36" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K36" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="37">
@@ -1716,28 +1716,28 @@
         <v>310</v>
       </c>
       <c r="D37" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E37" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F37" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G37" t="n">
         <v>0.001</v>
       </c>
       <c r="H37" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I37" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J37" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K37" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="38">
@@ -1751,28 +1751,28 @@
         <v>310</v>
       </c>
       <c r="D38" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E38" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F38" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G38" t="n">
         <v>0.001</v>
       </c>
       <c r="H38" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I38" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J38" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K38" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="39">
@@ -1786,28 +1786,28 @@
         <v>310</v>
       </c>
       <c r="D39" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E39" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F39" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G39" t="n">
         <v>0.001</v>
       </c>
       <c r="H39" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I39" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J39" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K39" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="40">
@@ -1821,28 +1821,28 @@
         <v>310</v>
       </c>
       <c r="D40" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E40" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F40" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G40" t="n">
         <v>0.001</v>
       </c>
       <c r="H40" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I40" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J40" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K40" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="41">
@@ -1856,28 +1856,28 @@
         <v>310</v>
       </c>
       <c r="D41" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E41" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F41" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G41" t="n">
         <v>0.001</v>
       </c>
       <c r="H41" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I41" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J41" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K41" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="42">
@@ -1891,28 +1891,28 @@
         <v>310</v>
       </c>
       <c r="D42" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E42" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F42" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G42" t="n">
         <v>0.001</v>
       </c>
       <c r="H42" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I42" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J42" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K42" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="43">
@@ -1926,28 +1926,28 @@
         <v>310</v>
       </c>
       <c r="D43" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E43" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F43" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G43" t="n">
         <v>0.001</v>
       </c>
       <c r="H43" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I43" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J43" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K43" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="44">
@@ -1961,28 +1961,28 @@
         <v>310</v>
       </c>
       <c r="D44" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E44" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F44" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G44" t="n">
         <v>0.001</v>
       </c>
       <c r="H44" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I44" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J44" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K44" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="45">
@@ -1996,28 +1996,28 @@
         <v>310</v>
       </c>
       <c r="D45" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E45" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F45" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G45" t="n">
         <v>0.001</v>
       </c>
       <c r="H45" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I45" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J45" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K45" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="46">
@@ -2031,28 +2031,28 @@
         <v>310</v>
       </c>
       <c r="D46" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E46" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F46" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G46" t="n">
         <v>0.001</v>
       </c>
       <c r="H46" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I46" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J46" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K46" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="47">
@@ -2066,28 +2066,28 @@
         <v>310</v>
       </c>
       <c r="D47" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E47" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F47" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G47" t="n">
         <v>0.001</v>
       </c>
       <c r="H47" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I47" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J47" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K47" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="48">
@@ -2101,28 +2101,28 @@
         <v>310</v>
       </c>
       <c r="D48" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E48" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F48" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G48" t="n">
         <v>0.001</v>
       </c>
       <c r="H48" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I48" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J48" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K48" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
     <row r="49">
@@ -2136,28 +2136,28 @@
         <v>310</v>
       </c>
       <c r="D49" t="n">
-        <v>0.1342517402857852</v>
+        <v>0.1342517402857851</v>
       </c>
       <c r="E49" t="n">
-        <v>0.1200124596983804</v>
+        <v>0.1200124596983803</v>
       </c>
       <c r="F49" t="n">
-        <v>9.428267071619871</v>
+        <v>9.428267071619864</v>
       </c>
       <c r="G49" t="n">
         <v>0.001</v>
       </c>
       <c r="H49" t="n">
-        <v>1128.927414843839</v>
+        <v>1128.927414843838</v>
       </c>
       <c r="I49" t="n">
         <v>8409.033748394333</v>
       </c>
       <c r="J49" t="n">
-        <v>2.028026433586267</v>
+        <v>2.028026433586264</v>
       </c>
       <c r="K49" t="n">
-        <v>1</v>
+        <v>1.785247080128419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>